<commit_message>
Criei a logica que executa uma busca nos contratos internos de acordo com o produto do contrato e utilizando o numero do contrato para acha-l0
</commit_message>
<xml_diff>
--- a/db/SOJA26.xlsx
+++ b/db/SOJA26.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10BCE490-0591-4725-ABC5-9AC5427ED62D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B724D250-AB33-41F9-9525-8BBC3C017C8A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2956,17 +2956,25 @@
   <dimension ref="A1:V278"/>
   <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.77734375" customWidth="1"/>
-    <col min="2" max="2" width="7.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="4.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="23.88671875" style="1" customWidth="1"/>
-    <col min="5" max="6" width="20.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="14.77734375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="6.77734375" style="2" customWidth="1"/>
-    <col min="10" max="16" width="60.77734375" style="1" customWidth="1"/>
-    <col min="17" max="20" width="8.77734375" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="60.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="39.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="49.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="60.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="59.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="59.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="20" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="11.77734375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="7.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">

</xml_diff>